<commit_message>
Fill demo gradebooks completely and restore avg/median charts with Std Dev as chart KPIs.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/demo-attendance.xlsx
+++ b/templates/demo-attendance.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:T18"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -415,6 +415,10 @@
     <col min="14" max="14" width="12.83203125" customWidth="1"/>
     <col min="15" max="15" width="12.83203125" customWidth="1"/>
     <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,7 +438,7 @@
         <v/>
       </c>
       <c r="F1" t="str">
-        <v>Progress Report</v>
+        <v>Unit 2</v>
       </c>
       <c r="G1" t="str">
         <v/>
@@ -446,7 +450,7 @@
         <v/>
       </c>
       <c r="J1" t="str">
-        <v>End of Term</v>
+        <v>Progress Report</v>
       </c>
       <c r="K1" t="str">
         <v/>
@@ -458,12 +462,24 @@
         <v/>
       </c>
       <c r="N1" t="str">
-        <v/>
+        <v>End of Term</v>
       </c>
       <c r="O1" t="str">
         <v/>
       </c>
       <c r="P1" t="str">
+        <v/>
+      </c>
+      <c r="Q1" t="str">
+        <v/>
+      </c>
+      <c r="R1" t="str">
+        <v/>
+      </c>
+      <c r="S1" t="str">
+        <v/>
+      </c>
+      <c r="T1" t="str">
         <v/>
       </c>
     </row>
@@ -508,12 +524,24 @@
         <v>D</v>
       </c>
       <c r="N2" t="str">
+        <v>A</v>
+      </c>
+      <c r="O2" t="str">
+        <v>B</v>
+      </c>
+      <c r="P2" t="str">
+        <v>C</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>D</v>
+      </c>
+      <c r="R2" t="str">
         <v>Attendance %</v>
       </c>
-      <c r="O2" t="str">
+      <c r="S2" t="str">
         <v>Homework %</v>
       </c>
-      <c r="P2" t="str">
+      <c r="T2" t="str">
         <v>EAL</v>
       </c>
     </row>
@@ -534,7 +562,7 @@
         <v>6</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G3">
         <v>6</v>
@@ -558,12 +586,24 @@
         <v>6</v>
       </c>
       <c r="N3">
+        <v>6</v>
+      </c>
+      <c r="O3">
+        <v>6</v>
+      </c>
+      <c r="P3">
+        <v>6</v>
+      </c>
+      <c r="Q3">
+        <v>6</v>
+      </c>
+      <c r="R3">
         <v>94</v>
       </c>
-      <c r="O3">
+      <c r="S3">
         <v>90</v>
       </c>
-      <c r="P3" t="str">
+      <c r="T3" t="str">
         <v>No</v>
       </c>
     </row>
@@ -584,7 +624,7 @@
         <v>6</v>
       </c>
       <c r="F4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4">
         <v>6</v>
@@ -608,12 +648,24 @@
         <v>6</v>
       </c>
       <c r="N4">
+        <v>7</v>
+      </c>
+      <c r="O4">
+        <v>6</v>
+      </c>
+      <c r="P4">
+        <v>6</v>
+      </c>
+      <c r="Q4">
+        <v>6</v>
+      </c>
+      <c r="R4">
         <v>95</v>
       </c>
-      <c r="O4">
+      <c r="S4">
         <v>92</v>
       </c>
-      <c r="P4" t="str">
+      <c r="T4" t="str">
         <v>No</v>
       </c>
     </row>
@@ -634,7 +686,7 @@
         <v>6</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G5">
         <v>6</v>
@@ -658,12 +710,24 @@
         <v>6</v>
       </c>
       <c r="N5">
+        <v>6</v>
+      </c>
+      <c r="O5">
+        <v>6</v>
+      </c>
+      <c r="P5">
+        <v>6</v>
+      </c>
+      <c r="Q5">
+        <v>6</v>
+      </c>
+      <c r="R5">
         <v>96</v>
       </c>
-      <c r="O5">
+      <c r="S5">
         <v>94</v>
       </c>
-      <c r="P5" t="str">
+      <c r="T5" t="str">
         <v>No</v>
       </c>
     </row>
@@ -684,7 +748,7 @@
         <v>6</v>
       </c>
       <c r="F6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G6">
         <v>6</v>
@@ -708,12 +772,24 @@
         <v>6</v>
       </c>
       <c r="N6">
+        <v>7</v>
+      </c>
+      <c r="O6">
+        <v>6</v>
+      </c>
+      <c r="P6">
+        <v>6</v>
+      </c>
+      <c r="Q6">
+        <v>6</v>
+      </c>
+      <c r="R6">
         <v>97</v>
       </c>
-      <c r="O6">
+      <c r="S6">
         <v>96</v>
       </c>
-      <c r="P6" t="str">
+      <c r="T6" t="str">
         <v>No</v>
       </c>
     </row>
@@ -734,7 +810,7 @@
         <v>6</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G7">
         <v>6</v>
@@ -758,12 +834,24 @@
         <v>6</v>
       </c>
       <c r="N7">
+        <v>6</v>
+      </c>
+      <c r="O7">
+        <v>6</v>
+      </c>
+      <c r="P7">
+        <v>6</v>
+      </c>
+      <c r="Q7">
+        <v>6</v>
+      </c>
+      <c r="R7">
         <v>98</v>
       </c>
-      <c r="O7">
+      <c r="S7">
         <v>98</v>
       </c>
-      <c r="P7" t="str">
+      <c r="T7" t="str">
         <v>No</v>
       </c>
     </row>
@@ -784,7 +872,7 @@
         <v>6</v>
       </c>
       <c r="F8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G8">
         <v>6</v>
@@ -808,12 +896,24 @@
         <v>6</v>
       </c>
       <c r="N8">
+        <v>7</v>
+      </c>
+      <c r="O8">
+        <v>6</v>
+      </c>
+      <c r="P8">
+        <v>6</v>
+      </c>
+      <c r="Q8">
+        <v>6</v>
+      </c>
+      <c r="R8">
         <v>94</v>
       </c>
-      <c r="O8">
+      <c r="S8">
         <v>90</v>
       </c>
-      <c r="P8" t="str">
+      <c r="T8" t="str">
         <v>No</v>
       </c>
     </row>
@@ -834,7 +934,7 @@
         <v>6</v>
       </c>
       <c r="F9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G9">
         <v>6</v>
@@ -858,12 +958,24 @@
         <v>6</v>
       </c>
       <c r="N9">
+        <v>6</v>
+      </c>
+      <c r="O9">
+        <v>6</v>
+      </c>
+      <c r="P9">
+        <v>6</v>
+      </c>
+      <c r="Q9">
+        <v>6</v>
+      </c>
+      <c r="R9">
         <v>95</v>
       </c>
-      <c r="O9">
+      <c r="S9">
         <v>92</v>
       </c>
-      <c r="P9" t="str">
+      <c r="T9" t="str">
         <v>No</v>
       </c>
     </row>
@@ -884,7 +996,7 @@
         <v>6</v>
       </c>
       <c r="F10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G10">
         <v>6</v>
@@ -908,12 +1020,24 @@
         <v>6</v>
       </c>
       <c r="N10">
+        <v>7</v>
+      </c>
+      <c r="O10">
+        <v>6</v>
+      </c>
+      <c r="P10">
+        <v>6</v>
+      </c>
+      <c r="Q10">
+        <v>6</v>
+      </c>
+      <c r="R10">
         <v>96</v>
       </c>
-      <c r="O10">
+      <c r="S10">
         <v>94</v>
       </c>
-      <c r="P10" t="str">
+      <c r="T10" t="str">
         <v>No</v>
       </c>
     </row>
@@ -934,7 +1058,7 @@
         <v>6</v>
       </c>
       <c r="F11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G11">
         <v>6</v>
@@ -958,12 +1082,24 @@
         <v>6</v>
       </c>
       <c r="N11">
+        <v>6</v>
+      </c>
+      <c r="O11">
+        <v>6</v>
+      </c>
+      <c r="P11">
+        <v>6</v>
+      </c>
+      <c r="Q11">
+        <v>6</v>
+      </c>
+      <c r="R11">
         <v>97</v>
       </c>
-      <c r="O11">
+      <c r="S11">
         <v>96</v>
       </c>
-      <c r="P11" t="str">
+      <c r="T11" t="str">
         <v>No</v>
       </c>
     </row>
@@ -984,7 +1120,7 @@
         <v>6</v>
       </c>
       <c r="F12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G12">
         <v>6</v>
@@ -1008,12 +1144,24 @@
         <v>6</v>
       </c>
       <c r="N12">
+        <v>7</v>
+      </c>
+      <c r="O12">
+        <v>6</v>
+      </c>
+      <c r="P12">
+        <v>6</v>
+      </c>
+      <c r="Q12">
+        <v>6</v>
+      </c>
+      <c r="R12">
         <v>98</v>
       </c>
-      <c r="O12">
+      <c r="S12">
         <v>98</v>
       </c>
-      <c r="P12" t="str">
+      <c r="T12" t="str">
         <v>No</v>
       </c>
     </row>
@@ -1034,7 +1182,7 @@
         <v>6</v>
       </c>
       <c r="F13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G13">
         <v>6</v>
@@ -1058,12 +1206,24 @@
         <v>6</v>
       </c>
       <c r="N13">
+        <v>6</v>
+      </c>
+      <c r="O13">
+        <v>6</v>
+      </c>
+      <c r="P13">
+        <v>6</v>
+      </c>
+      <c r="Q13">
+        <v>6</v>
+      </c>
+      <c r="R13">
         <v>94</v>
       </c>
-      <c r="O13">
+      <c r="S13">
         <v>90</v>
       </c>
-      <c r="P13" t="str">
+      <c r="T13" t="str">
         <v>No</v>
       </c>
     </row>
@@ -1108,12 +1268,24 @@
         <v>3</v>
       </c>
       <c r="N14">
+        <v>3</v>
+      </c>
+      <c r="O14">
+        <v>3</v>
+      </c>
+      <c r="P14">
+        <v>4</v>
+      </c>
+      <c r="Q14">
+        <v>3</v>
+      </c>
+      <c r="R14">
         <v>68</v>
       </c>
-      <c r="O14">
+      <c r="S14">
         <v>55</v>
       </c>
-      <c r="P14" t="str">
+      <c r="T14" t="str">
         <v>No</v>
       </c>
     </row>
@@ -1158,12 +1330,24 @@
         <v>3</v>
       </c>
       <c r="N15">
+        <v>3</v>
+      </c>
+      <c r="O15">
+        <v>3</v>
+      </c>
+      <c r="P15">
+        <v>4</v>
+      </c>
+      <c r="Q15">
+        <v>3</v>
+      </c>
+      <c r="R15">
         <v>70</v>
       </c>
-      <c r="O15">
+      <c r="S15">
         <v>59</v>
       </c>
-      <c r="P15" t="str">
+      <c r="T15" t="str">
         <v>Yes</v>
       </c>
     </row>
@@ -1208,12 +1392,24 @@
         <v>3</v>
       </c>
       <c r="N16">
+        <v>3</v>
+      </c>
+      <c r="O16">
+        <v>3</v>
+      </c>
+      <c r="P16">
+        <v>4</v>
+      </c>
+      <c r="Q16">
+        <v>3</v>
+      </c>
+      <c r="R16">
         <v>72</v>
       </c>
-      <c r="O16">
+      <c r="S16">
         <v>63</v>
       </c>
-      <c r="P16" t="str">
+      <c r="T16" t="str">
         <v>No</v>
       </c>
     </row>
@@ -1258,12 +1454,24 @@
         <v>3</v>
       </c>
       <c r="N17">
+        <v>3</v>
+      </c>
+      <c r="O17">
+        <v>3</v>
+      </c>
+      <c r="P17">
+        <v>4</v>
+      </c>
+      <c r="Q17">
+        <v>3</v>
+      </c>
+      <c r="R17">
         <v>74</v>
       </c>
-      <c r="O17">
+      <c r="S17">
         <v>67</v>
       </c>
-      <c r="P17" t="str">
+      <c r="T17" t="str">
         <v>No</v>
       </c>
     </row>
@@ -1308,18 +1516,30 @@
         <v>3</v>
       </c>
       <c r="N18">
+        <v>3</v>
+      </c>
+      <c r="O18">
+        <v>3</v>
+      </c>
+      <c r="P18">
+        <v>4</v>
+      </c>
+      <c r="Q18">
+        <v>3</v>
+      </c>
+      <c r="R18">
         <v>76</v>
       </c>
-      <c r="O18">
+      <c r="S18">
         <v>71</v>
       </c>
-      <c r="P18" t="str">
+      <c r="T18" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>